<commit_message>
chore: updated data to 0930 release
</commit_message>
<xml_diff>
--- a/sources/xlsx/4. 癌症發生率.xlsx
+++ b/sources/xlsx/4. 癌症發生率.xlsx
@@ -632,7 +632,7 @@
     <t>苗栗市</t>
   </si>
   <si>
-    <t>頭份鎮</t>
+    <t>頭份市</t>
   </si>
   <si>
     <t>苑裡鎮</t>
@@ -1154,7 +1154,7 @@
     <t>金沙鎮</t>
   </si>
   <si>
-    <t>金寧鎮</t>
+    <t>金寧鄉</t>
   </si>
   <si>
     <t>烈嶼鄉</t>

</xml_diff>